<commit_message>
NDC scenario edits to fix SAF implementation and passenger LDV std timelines
</commit_message>
<xml_diff>
--- a/InputData/trans/PVTStL/Policy Veh Types Subject to LCFS.xlsx
+++ b/InputData/trans/PVTStL/Policy Veh Types Subject to LCFS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\PVTStL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A8B7640-3F18-4F5C-A9FF-A8B089B6F820}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FF4771-DE8E-4431-9365-19D37BF6EB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>Source:</t>
   </si>
@@ -80,10 +80,13 @@
     <t>(Boolean)</t>
   </si>
   <si>
-    <t>Based on the California LCFS, we choose to exempt aircraft.</t>
-  </si>
-  <si>
     <t>PVTStL Policy Vehicle Types Subject to LCFS</t>
+  </si>
+  <si>
+    <t>We configure this file to apply only to aviation in order to represent</t>
+  </si>
+  <si>
+    <t>policy support for sustainable aviation fuel.</t>
   </si>
 </sst>
 </file>
@@ -440,15 +443,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B16"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -456,54 +459,59 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B4" s="2">
         <v>2015</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
       <c r="B7" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A16" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>
@@ -518,14 +526,14 @@
     <tabColor theme="3"/>
   </sheetPr>
   <dimension ref="A1:C7"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.140625" customWidth="1"/>
-    <col min="2" max="2" width="15.140625" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" customWidth="1"/>
+    <col min="1" max="1" width="14.1796875" customWidth="1"/>
+    <col min="2" max="2" width="15.1796875" customWidth="1"/>
+    <col min="3" max="3" width="13.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>18</v>
       </c>
@@ -536,7 +544,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -547,7 +555,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -558,7 +566,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -569,7 +577,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -580,18 +588,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>6</v>
       </c>
       <c r="B6">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>7</v>
       </c>

</xml_diff>

<commit_message>
Add shipping back into vehicle types covered by LCFS
</commit_message>
<xml_diff>
--- a/InputData/trans/PVTStL/Policy Veh Types Subject to LCFS.xlsx
+++ b/InputData/trans/PVTStL/Policy Veh Types Subject to LCFS.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\trans\PVTStL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91FF4771-DE8E-4431-9365-19D37BF6EB64}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7667BF24-AF7B-44D4-86C9-83BEB73ADAEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -83,10 +83,10 @@
     <t>PVTStL Policy Vehicle Types Subject to LCFS</t>
   </si>
   <si>
-    <t>We configure this file to apply only to aviation in order to represent</t>
-  </si>
-  <si>
-    <t>policy support for sustainable aviation fuel.</t>
+    <t>We configure this file to apply only to aviation and shipping in order to represent</t>
+  </si>
+  <si>
+    <t>policy support for sustainable aviation and shipping fuel.</t>
   </si>
 </sst>
 </file>
@@ -593,10 +593,10 @@
         <v>6</v>
       </c>
       <c r="B6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C6">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Adds psgr vehicles to LCFS
</commit_message>
<xml_diff>
--- a/InputData/trans/PVTStL/Policy Veh Types Subject to LCFS.xlsx
+++ b/InputData/trans/PVTStL/Policy Veh Types Subject to LCFS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanOBrien\Models\EPS\US\eps-us\InputData\trans\PVTStL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFFDD382-3D5A-4AA8-96B4-6347108D931A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D9DDAF-76D6-41CF-A17D-78ADD389977F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2820" yWindow="1110" windowWidth="23520" windowHeight="15450" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="21120" windowHeight="14760" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -549,7 +549,7 @@
         <v>2</v>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C2">
         <v>1</v>
@@ -560,7 +560,7 @@
         <v>3</v>
       </c>
       <c r="B3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C3">
         <v>1</v>

</xml_diff>